<commit_message>
5262 - MOQ Table import backend
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/MOQTableSSC.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/MOQTableSSC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5186B8CF-2C3F-4A70-8192-354591EDC35E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAADD539-BEDB-40AA-B034-4F397B15DCC2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1110" yWindow="-120" windowWidth="27810" windowHeight="16440" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
   </bookViews>
   <sheets>
     <sheet name="MOQ Tables" sheetId="1" r:id="rId1"/>
@@ -625,13 +625,13 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="42" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="41.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="42" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41.140625" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="57.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="60.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="26.140625" style="2" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
PROPH-1246: Add Period Of Performance Month to SSC.
</commit_message>
<xml_diff>
--- a/GenBOE/GenBOE.Web/Templates/Export/MOQTableSSC.xlsx
+++ b/GenBOE/GenBOE.Web/Templates/Export/MOQTableSSC.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ranzalon\Source\repos\IES\GenBOE\GenBOE.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\GenBOE.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAADD539-BEDB-40AA-B034-4F397B15DCC2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258EDB6D-AB4B-4563-856D-409F479859E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
+    <workbookView xWindow="22305" yWindow="15" windowWidth="34035" windowHeight="21570" xr2:uid="{F2BDE59F-50D5-4F91-B73E-5DFBD476F53C}"/>
   </bookViews>
   <sheets>
     <sheet name="MOQ Tables" sheetId="1" r:id="rId1"/>
     <sheet name="Option Lists" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOQ Tables'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MOQ Tables'!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -97,7 +97,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Table Name</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t>Monthly</t>
+  </si>
+  <si>
+    <t>Period of Performance (PoP): Months</t>
   </si>
 </sst>
 </file>
@@ -290,7 +293,7 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -300,6 +303,9 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="5" fillId="7" borderId="1" xfId="7" applyNumberFormat="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="genBOE" xfId="7" xr:uid="{3E4869EB-5B79-4DE7-855F-A2B8CADB72D2}"/>
@@ -621,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C581C636-3424-4611-9D2C-375716778AB5}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
@@ -632,12 +638,13 @@
     <col min="6" max="6" width="42" style="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="42" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="41.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="57.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="60.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="26.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="39.140625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="57.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="60.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.140625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -662,21 +669,24 @@
       <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="F2" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1" xr:uid="{7D4A90C3-D4CB-40BE-BC1C-2D75CA06857E}"/>
+  <autoFilter ref="A1:K1" xr:uid="{7D4A90C3-D4CB-40BE-BC1C-2D75CA06857E}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <headerFooter>

</xml_diff>